<commit_message>
feat: recover lost equipment only through found and returned
</commit_message>
<xml_diff>
--- a/sample_data/mapatz-full-recovery-sample.xlsx
+++ b/sample_data/mapatz-full-recovery-sample.xlsx
@@ -1178,16 +1178,16 @@
     <t>2026-01-01T10:16:00.000Z</t>
   </si>
   <si>
-    <t>unmarked_lost</t>
-  </si>
-  <si>
-    <t>נמצא בחיפוש בציוד</t>
+    <t>found_returned</t>
+  </si>
+  <si>
+    <t>ציוד אבוד נמצא והוחזר למחסן</t>
   </si>
   <si>
     <t>2026-01-01T10:17:00.000Z</t>
   </si>
   <si>
-    <t>הוחזר תקין לאחר איתור</t>
+    <t>החזרה רגילה של היחידה שנותרה בהשאלה</t>
   </si>
   <si>
     <t>2026-01-01T10:18:00.000Z</t>
@@ -1939,7 +1939,7 @@
   </sheetData>
   <autoFilter ref="A1:B1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3717,7 +3717,7 @@
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3764,7 +3764,7 @@
   </sheetData>
   <autoFilter ref="A1:B1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -5982,7 +5982,7 @@
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -6257,7 +6257,7 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -9104,7 +9104,7 @@
         <v>178</v>
       </c>
       <c r="E139">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F139">
         <v>135</v>
@@ -9876,7 +9876,7 @@
         <v>178</v>
       </c>
       <c r="E171">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F171">
         <v>167</v>
@@ -10648,7 +10648,7 @@
         <v>178</v>
       </c>
       <c r="E203">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F203">
         <v>199</v>
@@ -11118,7 +11118,7 @@
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -11232,7 +11232,7 @@
   </sheetData>
   <autoFilter ref="A1:D1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -12101,6 +12101,6 @@
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add radio custody tracking
</commit_message>
<xml_diff>
--- a/sample_data/mapatz-full-recovery-sample.xlsx
+++ b/sample_data/mapatz-full-recovery-sample.xlsx
@@ -12,13 +12,15 @@
     <sheet sheetId="6" name="Recovery Events" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="Unresolved Damage" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="Consumables Usage" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Recovery Radio Fleet" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="Recovery Radios" state="visible" r:id="rId13"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2506" uniqueCount="798">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2511" uniqueCount="803">
   <si>
     <t>Name</t>
   </si>
@@ -2412,6 +2414,21 @@
   </si>
   <si>
     <t>Left</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>Number</t>
+  </si>
+  <si>
+    <t>Holder</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Lost</t>
   </si>
 </sst>
 </file>
@@ -2837,6 +2854,31 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>799</v>
+      </c>
+      <c r="B1" t="s">
+        <v>800</v>
+      </c>
+      <c r="C1" t="s">
+        <v>801</v>
+      </c>
+      <c r="D1" t="s">
+        <v>802</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H73"/>
@@ -18792,4 +18834,25 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add full record deletion
</commit_message>
<xml_diff>
--- a/sample_data/mapatz-full-recovery-sample.xlsx
+++ b/sample_data/mapatz-full-recovery-sample.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2740" uniqueCount="809">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2745" uniqueCount="814">
   <si>
     <t>Name</t>
   </si>
@@ -2449,6 +2449,21 @@
   </si>
   <si>
     <t>Outstanding</t>
+  </si>
+  <si>
+    <t>Next Item Code</t>
+  </si>
+  <si>
+    <t>Next Item ID</t>
+  </si>
+  <si>
+    <t>Next Borrower ID</t>
+  </si>
+  <si>
+    <t>Next Location ID</t>
+  </si>
+  <si>
+    <t>Next Event ID</t>
   </si>
 </sst>
 </file>
@@ -5413,28 +5428,58 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>809</v>
+      </c>
+      <c r="C1" t="s">
+        <v>810</v>
+      </c>
+      <c r="D1" t="s">
+        <v>811</v>
+      </c>
+      <c r="E1" t="s">
+        <v>812</v>
+      </c>
+      <c r="F1" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>483</v>
       </c>
+      <c r="B2">
+        <v>236</v>
+      </c>
+      <c r="C2">
+        <v>73</v>
+      </c>
+      <c r="D2">
+        <v>13</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>484</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Update sample radio fleet
</commit_message>
<xml_diff>
--- a/sample_data/mapatz-full-recovery-sample.xlsx
+++ b/sample_data/mapatz-full-recovery-sample.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2745" uniqueCount="814">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2775" uniqueCount="824">
   <si>
     <t>Name</t>
   </si>
@@ -2443,6 +2443,36 @@
   </si>
   <si>
     <t>Team</t>
+  </si>
+  <si>
+    <t>מתנדב מד״א</t>
+  </si>
+  <si>
+    <t>מד״א</t>
+  </si>
+  <si>
+    <t>צוות הפקה</t>
+  </si>
+  <si>
+    <t>במה</t>
+  </si>
+  <si>
+    <t>מאנקי</t>
+  </si>
+  <si>
+    <t>לוגיסטיקה</t>
+  </si>
+  <si>
+    <t>נועה כהן</t>
+  </si>
+  <si>
+    <t>רפואה</t>
+  </si>
+  <si>
+    <t>עובד מד״א</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>Checkout ID</t>
@@ -2891,7 +2921,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2906,6 +2936,216 @@
       </c>
       <c r="D1" t="s">
         <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>807</v>
+      </c>
+      <c r="C2" t="s">
+        <v>808</v>
+      </c>
+      <c r="D2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>809</v>
+      </c>
+      <c r="C3" t="s">
+        <v>810</v>
+      </c>
+      <c r="D3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>811</v>
+      </c>
+      <c r="C4" t="s">
+        <v>812</v>
+      </c>
+      <c r="D4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>813</v>
+      </c>
+      <c r="C5" t="s">
+        <v>814</v>
+      </c>
+      <c r="D5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>815</v>
+      </c>
+      <c r="C6" t="s">
+        <v>808</v>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>816</v>
+      </c>
+      <c r="D7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>816</v>
+      </c>
+      <c r="D8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>816</v>
+      </c>
+      <c r="D9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>816</v>
+      </c>
+      <c r="D10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" t="s">
+        <v>816</v>
+      </c>
+      <c r="D11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" t="s">
+        <v>816</v>
+      </c>
+      <c r="D12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" t="s">
+        <v>816</v>
+      </c>
+      <c r="D13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>816</v>
+      </c>
+      <c r="D14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>816</v>
+      </c>
+      <c r="D15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>816</v>
+      </c>
+      <c r="D16" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2921,7 +3161,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>807</v>
+        <v>817</v>
       </c>
       <c r="B1" t="s">
         <v>5</v>
@@ -2936,7 +3176,7 @@
         <v>107</v>
       </c>
       <c r="F1" t="s">
-        <v>808</v>
+        <v>818</v>
       </c>
       <c r="G1" t="s">
         <v>113</v>
@@ -5442,19 +5682,19 @@
         <v>114</v>
       </c>
       <c r="B1" t="s">
-        <v>809</v>
+        <v>819</v>
       </c>
       <c r="C1" t="s">
-        <v>810</v>
+        <v>820</v>
       </c>
       <c r="D1" t="s">
-        <v>811</v>
+        <v>821</v>
       </c>
       <c r="E1" t="s">
-        <v>812</v>
+        <v>822</v>
       </c>
       <c r="F1" t="s">
-        <v>813</v>
+        <v>823</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -22547,7 +22787,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Default radio fleet and sample data to 40 radios
</commit_message>
<xml_diff>
--- a/sample_data/mapatz-full-recovery-sample.xlsx
+++ b/sample_data/mapatz-full-recovery-sample.xlsx
@@ -2921,7 +2921,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -3145,6 +3145,356 @@
         <v>816</v>
       </c>
       <c r="D16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C17" t="str"/>
+      <c r="D17" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C18" t="str"/>
+      <c r="D18" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C19" t="str"/>
+      <c r="D19" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C20" t="str"/>
+      <c r="D20" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C21" t="str"/>
+      <c r="D21" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C22" t="str"/>
+      <c r="D22" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C23" t="str"/>
+      <c r="D23" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C24" t="str"/>
+      <c r="D24" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C25" t="str"/>
+      <c r="D25" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C26" t="str"/>
+      <c r="D26" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C27" t="str"/>
+      <c r="D27" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C28" t="str"/>
+      <c r="D28" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C29" t="str"/>
+      <c r="D29" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C30" t="str"/>
+      <c r="D30" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C31" t="str"/>
+      <c r="D31" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C32" t="str"/>
+      <c r="D32" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C33" t="str"/>
+      <c r="D33" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C34" t="str"/>
+      <c r="D34" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C35" t="str"/>
+      <c r="D35" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C36" t="str"/>
+      <c r="D36" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C37" t="str"/>
+      <c r="D37" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C38" t="str"/>
+      <c r="D38" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C39" t="str"/>
+      <c r="D39" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C40" t="str"/>
+      <c r="D40" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>צוללת</t>
+        </is>
+      </c>
+      <c r="C41" t="str"/>
+      <c r="D41" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -22787,7 +23137,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>15</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: add matching item notes to sample workbook
</commit_message>
<xml_diff>
--- a/sample_data/mapatz-full-recovery-sample.xlsx
+++ b/sample_data/mapatz-full-recovery-sample.xlsx
@@ -4477,8 +4477,10 @@
       <c r="G2">
         <v>117</v>
       </c>
-      <c r="H2" t="s">
-        <v>15</v>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>לסגור בסיום</t>
+        </is>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -4503,8 +4505,10 @@
       <c r="G3">
         <v>121</v>
       </c>
-      <c r="H3" t="s">
-        <v>15</v>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>קופסה כחולה</t>
+        </is>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -5455,8 +5459,10 @@
       <c r="G41">
         <v>6</v>
       </c>
-      <c r="H41" t="s">
-        <v>15</v>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>ידית אדומה</t>
+        </is>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
@@ -5524,8 +5530,10 @@
       <c r="G44">
         <v>11</v>
       </c>
-      <c r="H44" t="s">
-        <v>15</v>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>להחזיר נקי</t>
+        </is>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -6030,8 +6038,10 @@
       <c r="G66">
         <v>3</v>
       </c>
-      <c r="H66" t="s">
-        <v>15</v>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>לגלגל בסיום</t>
+        </is>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
@@ -6076,8 +6086,10 @@
       <c r="G68">
         <v>8</v>
       </c>
-      <c r="H68" t="s">
-        <v>15</v>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>סט משותף</t>
+        </is>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
@@ -6260,8 +6272,10 @@
       <c r="G76">
         <v>3</v>
       </c>
-      <c r="H76" t="s">
-        <v>15</v>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>ידית אדומה</t>
+        </is>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
@@ -6329,8 +6343,10 @@
       <c r="G79">
         <v>1</v>
       </c>
-      <c r="H79" t="s">
-        <v>15</v>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>להחזיר נקי</t>
+        </is>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
@@ -6651,8 +6667,10 @@
       <c r="G93">
         <v>3</v>
       </c>
-      <c r="H93" t="s">
-        <v>15</v>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>לגלגל בסיום</t>
+        </is>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.25">
@@ -6871,8 +6889,10 @@
       <c r="O2">
         <v>485</v>
       </c>
-      <c r="P2" t="s">
-        <v>15</v>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>לסגור בסיום</t>
+        </is>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
@@ -6918,8 +6938,10 @@
       <c r="O3">
         <v>485</v>
       </c>
-      <c r="P3" t="s">
-        <v>15</v>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>לסגור בסיום</t>
+        </is>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -6968,8 +6990,10 @@
       <c r="O4">
         <v>487</v>
       </c>
-      <c r="P4" t="s">
-        <v>15</v>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>קופסה כחולה</t>
+        </is>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -7018,8 +7042,10 @@
       <c r="O5">
         <v>487</v>
       </c>
-      <c r="P5" t="s">
-        <v>15</v>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>קופסה כחולה</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -8882,8 +8908,10 @@
       <c r="O43">
         <v>489</v>
       </c>
-      <c r="P43" t="s">
-        <v>15</v>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>ידית אדומה</t>
+        </is>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
@@ -8929,8 +8957,10 @@
       <c r="O44">
         <v>489</v>
       </c>
-      <c r="P44" t="s">
-        <v>15</v>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>ידית אדומה</t>
+        </is>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
@@ -9117,8 +9147,10 @@
       <c r="O48">
         <v>493</v>
       </c>
-      <c r="P48" t="s">
-        <v>15</v>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>להחזיר נקי</t>
+        </is>
       </c>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
@@ -9164,8 +9196,10 @@
       <c r="O49">
         <v>493</v>
       </c>
-      <c r="P49" t="s">
-        <v>15</v>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>להחזיר נקי</t>
+        </is>
       </c>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
@@ -10198,8 +10232,10 @@
       <c r="O71">
         <v>423</v>
       </c>
-      <c r="P71" t="s">
-        <v>15</v>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>לגלגל בסיום</t>
+        </is>
       </c>
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.25">
@@ -10292,8 +10328,10 @@
       <c r="O73">
         <v>497</v>
       </c>
-      <c r="P73" t="s">
-        <v>15</v>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>סט משותף</t>
+        </is>
       </c>
     </row>
     <row r="74" spans="1:16" x14ac:dyDescent="0.25">
@@ -10339,8 +10377,10 @@
       <c r="O74">
         <v>497</v>
       </c>
-      <c r="P74" t="s">
-        <v>15</v>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>סט משותף</t>
+        </is>
       </c>
     </row>
     <row r="75" spans="1:16" x14ac:dyDescent="0.25">

</xml_diff>